<commit_message>
Update v6 Excel file with Growth Tendency data
</commit_message>
<xml_diff>
--- a/rpg-performance-tracker-v6.xlsx
+++ b/rpg-performance-tracker-v6.xlsx
@@ -1,39 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD17475-617C-44AA-9D53-2711F6C22FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="4" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="คำแนะนำการใช้งาน" sheetId="1" r:id="rId1"/>
-    <sheet name="ประเมินผลทีม" sheetId="2" r:id="rId2"/>
-    <sheet name="เกณฑ์ประเมินแบบละเอียด" sheetId="3" r:id="rId3"/>
-    <sheet name="Archetypes Guide V2" sheetId="4" r:id="rId4"/>
-    <sheet name="Stats Definition V2" sheetId="5" r:id="rId5"/>
-    <sheet name="สรุปผลการประเมิน" sheetId="6" r:id="rId6"/>
+    <sheet sheetId="1" name="คำแนะนำการใช้งาน" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="ประเมินผลทีม" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="เกณฑ์ประเมินแบบละเอียด" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Archetypes Guide V2" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Stats Definition V2" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="สรุปผลการประเมิน" state="visible" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="348">
   <si>
     <t>คู่มือและระบบบันทึกคะแนน RPG Status Framework (ฉบับอัปเดตเกณฑ์ใหม่)</t>
   </si>
@@ -167,79 +153,79 @@
     <t>จุดที่ควรพัฒนา</t>
   </si>
   <si>
-    <t>STR1
+    <t xml:space="preserve">STR1
 เด็ดขาด</t>
   </si>
   <si>
-    <t>STR2
+    <t xml:space="preserve">STR2
 ปิดเคสยาก</t>
   </si>
   <si>
-    <t>STR3
+    <t xml:space="preserve">STR3
 คุมผู้รับเหมา</t>
   </si>
   <si>
-    <t>AGI1
+    <t xml:space="preserve">AGI1
 ตอบสนองไว</t>
   </si>
   <si>
-    <t>AGI2
+    <t xml:space="preserve">AGI2
 เหตุฉุกเฉิน</t>
   </si>
   <si>
-    <t>AGI3
+    <t xml:space="preserve">AGI3
 ปรับยืดหยุ่น</t>
   </si>
   <si>
-    <t>DEX1
+    <t xml:space="preserve">DEX1
 ข้อมูลแม่น</t>
   </si>
   <si>
-    <t>DEX2
+    <t xml:space="preserve">DEX2
 ตรวจละเอียด</t>
   </si>
   <si>
-    <t>DEX3
+    <t xml:space="preserve">DEX3
 มาตรฐานSLA</t>
   </si>
   <si>
-    <t>INT1
+    <t xml:space="preserve">INT1
 วิเคราะห์ราก</t>
   </si>
   <si>
-    <t>INT2
+    <t xml:space="preserve">INT2
 ความรู้ระบบ</t>
   </si>
   <si>
-    <t>INT3
+    <t xml:space="preserve">INT3
 แผนเชิงป้องกัน</t>
   </si>
   <si>
-    <t>INT4
+    <t xml:space="preserve">INT4
 คิดสร้างสรรค์</t>
   </si>
   <si>
-    <t>CON1
+    <t xml:space="preserve">CON1
 คุมอารมณ์</t>
   </si>
   <si>
-    <t>CON2
+    <t xml:space="preserve">CON2
 ทนแรงกดดัน</t>
   </si>
   <si>
-    <t>CON3
+    <t xml:space="preserve">CON3
 เข้าใจลูกค้า</t>
   </si>
   <si>
-    <t>SEN1
+    <t xml:space="preserve">SEN1
 บริหารคิว</t>
   </si>
   <si>
-    <t>SEN2
+    <t xml:space="preserve">SEN2
 เทคโนโลยีตามงาน</t>
   </si>
   <si>
-    <t>SEN3
+    <t xml:space="preserve">SEN3
 เทคโนโลยีลดขั้นตอน</t>
   </si>
   <si>
@@ -273,14 +259,14 @@
     <t>ระดับสูง (7-8) / ระดับเชี่ยวชาญ (9-10)</t>
   </si>
   <si>
-    <t>STR (Strength)
+    <t xml:space="preserve">STR (Strength)
 พลังผลักดันหน้างาน</t>
   </si>
   <si>
     <t>STR1</t>
   </si>
   <si>
-    <t>ความเด็ดขาดในการแก้ปัญหา
+    <t xml:space="preserve">ความเด็ดขาดในการแก้ปัญหา
 (Decision Making)</t>
   </si>
   <si>
@@ -299,7 +285,7 @@
     <t>STR2</t>
   </si>
   <si>
-    <t>อัตราการปิดเคสยาก
+    <t xml:space="preserve">อัตราการปิดเคสยาก
 (Case Closure)</t>
   </si>
   <si>
@@ -318,7 +304,7 @@
     <t>STR3</t>
   </si>
   <si>
-    <t>การควบคุมผลงานช่าง/ผู้รับเหมา
+    <t xml:space="preserve">การควบคุมผลงานช่าง/ผู้รับเหมา
 (Site &amp; Subcontractor Control)</t>
   </si>
   <si>
@@ -334,14 +320,14 @@
     <t>ควบคุมคุณภาพงานซ่อมของผู้รับเหมาได้เนี๊ยบระดับแชมป์ ปรับเปลี่ยนแผนคุมงานเมื่อเกิดเหตุไม่คาดคิดได้ฉลุย</t>
   </si>
   <si>
-    <t>AGI (Agility)
+    <t xml:space="preserve">AGI (Agility)
 ความรวดเร็วและปรับตัว</t>
   </si>
   <si>
     <t>AGI1</t>
   </si>
   <si>
-    <t>ความรวดเร็วในการตอบสนอง
+    <t xml:space="preserve">ความรวดเร็วในการตอบสนอง
 (First Response)</t>
   </si>
   <si>
@@ -378,7 +364,7 @@
     <t>AGI3</t>
   </si>
   <si>
-    <t>ความยืดหยุ่นในการปรับแผน
+    <t xml:space="preserve">ความยืดหยุ่นในการปรับแผน
 (Adaptability)</t>
   </si>
   <si>
@@ -394,14 +380,14 @@
     <t>มองหาแผนสำรอง (Plan B) คู่อยู่เสมอ ปรับทีมตอบสนองได้แบบ Real-time โดยประสิทธิภาพโดยรวมไม่ลด</t>
   </si>
   <si>
-    <t>DEX (Dexterity)
+    <t xml:space="preserve">DEX (Dexterity)
 ความแม่นยำและเป๊ะ</t>
   </si>
   <si>
     <t>DEX1</t>
   </si>
   <si>
-    <t>ความถูกต้องของข้อมูลและงานเอกสาร
+    <t xml:space="preserve">ความถูกต้องของข้อมูลและงานเอกสาร
 (Data &amp; Document Accuracy)</t>
   </si>
   <si>
@@ -420,7 +406,7 @@
     <t>DEX2</t>
   </si>
   <si>
-    <t>ความละเอียดในการตรวจงาน
+    <t xml:space="preserve">ความละเอียดในการตรวจงาน
 (QC Precision)</t>
   </si>
   <si>
@@ -439,7 +425,7 @@
     <t>DEX3</t>
   </si>
   <si>
-    <t>การรักษามาตรฐานเวลา
+    <t xml:space="preserve">การรักษามาตรฐานเวลา
 (SLA &amp; Compliance)</t>
   </si>
   <si>
@@ -455,14 +441,14 @@
     <t>รักษาอัตรา 100% SLA ยอดเยี่ยมอย่างต่อเนื่อง ปรับขั้นตอนที่ซ้ำซ้อนให้ทีมส่งงานได้เร็วขึ้นอย่างยั่งยืน</t>
   </si>
   <si>
-    <t>INT (Intelligence)
+    <t xml:space="preserve">INT (Intelligence)
 การวิเคราะห์และกลยุทธ์</t>
   </si>
   <si>
     <t>INT1</t>
   </si>
   <si>
-    <t>การวิเคราะห์หาสาเหตุปัญหาที่ถูกต้อง
+    <t xml:space="preserve">การวิเคราะห์หาสาเหตุปัญหาที่ถูกต้อง
 (Accurate Root Cause Analysis)</t>
   </si>
   <si>
@@ -481,7 +467,7 @@
     <t>INT2</t>
   </si>
   <si>
-    <t>ความรู้ความเข้าใจงานระบบในองค์กร
+    <t xml:space="preserve">ความรู้ความเข้าใจงานระบบในองค์กร
 (System &amp; Domain Knowledge)</t>
   </si>
   <si>
@@ -500,7 +486,7 @@
     <t>INT3</t>
   </si>
   <si>
-    <t>การวางแผนและการแก้ปัญหาเชิงประยุกต์
+    <t xml:space="preserve">การวางแผนและการแก้ปัญหาเชิงประยุกต์
 (Preventive &amp; Creative Solving)</t>
   </si>
   <si>
@@ -516,14 +502,14 @@
     <t>ออกแบบระบบป้องกันวิกฤตขั้นสูง และคิดค้นนวัตกรรมการบริการหรือเทคนิคเจรจาใหม่ๆ ที่ไม่มีในตำรา</t>
   </si>
   <si>
-    <t>CON (Constitution)
+    <t xml:space="preserve">CON (Constitution)
 ความอดทนและควบคุมจิตใจ</t>
   </si>
   <si>
     <t>CON1</t>
   </si>
   <si>
-    <t>การควบคุมอารมณ์และสติ
+    <t xml:space="preserve">การควบคุมอารมณ์และสติ
 (Emotional Control)</t>
   </si>
   <si>
@@ -542,7 +528,7 @@
     <t>CON2</t>
   </si>
   <si>
-    <t>ความสม่ำเสมอในสภาวะกดดัน
+    <t xml:space="preserve">ความสม่ำเสมอในสภาวะกดดัน
 (Burnout Resilience)</t>
   </si>
   <si>
@@ -561,7 +547,7 @@
     <t>CON3</t>
   </si>
   <si>
-    <t>ทักษะการรับฟังและเข้าอกเข้าใจ
+    <t xml:space="preserve">ทักษะการรับฟังและเข้าอกเข้าใจ
 (Customer Empathy)</t>
   </si>
   <si>
@@ -577,14 +563,14 @@
     <t>สร้างความประทับใจระดับตำนาน (Customer Delight) ลูกค้าส่งจดหมายชื่นชมหรือเจาะจงชมเชยเป็นรายบุคคล</t>
   </si>
   <si>
-    <t>SEN (Sensibility)
+    <t xml:space="preserve">SEN (Sensibility)
 การบริหารจัดการและเทคโนโลยี</t>
   </si>
   <si>
     <t>SEN1</t>
   </si>
   <si>
-    <t>การบริหารจัดการคิวงานและทรัพยากร
+    <t xml:space="preserve">การบริหารจัดการคิวงานและทรัพยากร
 (Task &amp; Resource Management)</t>
   </si>
   <si>
@@ -603,7 +589,7 @@
     <t>SEN2</t>
   </si>
   <si>
-    <t>การใช้เทคโนโลยีติดตามสถานะงาน
+    <t xml:space="preserve">การใช้เทคโนโลยีติดตามสถานะงาน
 (Systematic Tracking &amp; Monitoring)</t>
   </si>
   <si>
@@ -622,7 +608,7 @@
     <t>SEN3</t>
   </si>
   <si>
-    <t>การประยุกต์ใช้เทคโนโลยีเพื่อลดขั้นตอน
+    <t xml:space="preserve">การประยุกต์ใช้เทคโนโลยีเพื่อลดขั้นตอน
 (Process Automation)</t>
   </si>
   <si>
@@ -1119,43 +1105,38 @@
   </si>
   <si>
     <t>คำอธิบาย</t>
-  </si>
-  <si>
-    <t>AGI+STR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="16"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1167,25 +1148,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="2" tint="-0.0999786370433668"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1197,13 +1178,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
+        <fgColor theme="8" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1270,8 +1251,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1339,22 +1321,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1693,22 +1659,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="29" t="s">
+    <row r="1" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1716,7 +1682,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1724,7 +1690,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1732,7 +1698,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1740,7 +1706,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1748,7 +1714,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1756,7 +1722,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1764,12 +1730,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1777,7 +1743,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1785,7 +1751,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1793,7 +1759,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1801,7 +1767,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1809,12 +1775,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1822,7 +1788,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1830,7 +1796,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1847,48 +1813,48 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AC25"/>
-  <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.73046875" customWidth="1"/>
     <col min="2" max="2" width="18.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="29" t="s">
+    <row r="1" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-    </row>
-    <row r="2" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1977,7 +1943,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C3">
         <f t="shared" ref="C3:C25" si="0">ROUND(ROUND(AVERAGE(K3:M3), 1), 0)</f>
         <v>7</v>
@@ -2068,7 +2034,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C4">
         <f>ROUND(ROUND(AVERAGE(K4:M4), 1), 0)</f>
         <v>5</v>
@@ -2159,7 +2125,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C5">
         <f>ROUND(ROUND(AVERAGE(K5:M5), 1), 0)</f>
         <v>6</v>
@@ -2250,7 +2216,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -2347,7 +2313,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2381,7 +2347,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="8" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C8" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2415,7 +2381,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="9" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2449,7 +2415,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2483,7 +2449,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="11" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C11" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2517,7 +2483,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2551,7 +2517,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C13" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2585,7 +2551,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C14" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2619,7 +2585,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C15" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2653,7 +2619,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C16" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2687,7 +2653,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C17" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2721,7 +2687,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2755,7 +2721,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="19" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C19" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2789,7 +2755,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C20" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2823,7 +2789,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="21" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C21" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2857,7 +2823,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C22" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2891,7 +2857,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="23" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C23" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2925,7 +2891,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="24" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C24" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -2959,7 +2925,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="25" spans="3:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C25" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
@@ -3002,449 +2968,448 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="70.53125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="70.53125" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="45.9296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.53125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="70.53125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="76.796875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="95.6640625" style="2" customWidth="1"/>
-    <col min="6" max="7" width="70.53125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="70.53125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="70.53125" style="1"/>
+    <col min="1" max="1" width="45.9296875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.53125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="70.53125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="76.796875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="95.6640625" style="3" customWidth="1"/>
+    <col min="6" max="7" width="70.53125" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="70.53125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="25" t="s">
+    <row r="3" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="25"/>
-      <c r="B4" s="3" t="s">
+    <row r="4" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="25"/>
-      <c r="B5" s="3" t="s">
+    <row r="5" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="26" t="s">
+    <row r="6" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="26"/>
-      <c r="B7" s="5" t="s">
+    <row r="7" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="26"/>
-      <c r="B8" s="5" t="s">
+    <row r="8" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="27" t="s">
+    <row r="9" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="27"/>
-      <c r="B10" s="7" t="s">
+    <row r="10" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="27"/>
-      <c r="B11" s="7" t="s">
+    <row r="11" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="9" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="28" t="s">
+    <row r="12" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="11" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="28"/>
-      <c r="B13" s="9" t="s">
+    <row r="13" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="11" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="28"/>
-      <c r="B14" s="9" t="s">
+    <row r="14" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="11" t="s">
+    <row r="15" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="13" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="11" t="s">
+    <row r="16" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="11" t="s">
+    <row r="17" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="13" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="13" t="s">
+    <row r="18" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="G18" s="14" t="s">
+      <c r="G18" s="15" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="13" t="s">
+    <row r="19" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="G19" s="14" t="s">
+      <c r="G19" s="15" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="13" t="s">
+    <row r="20" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="G20" s="14" t="s">
+      <c r="G20" s="15" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3461,629 +3426,628 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E36"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="80" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="80" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43.9296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.19921875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="69.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="50.3984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="9" style="2" customWidth="1"/>
+    <col min="2" max="2" width="43.9296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.19921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="69.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="50.3984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="19" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="1">
+    <row r="2" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="1">
+    <row r="3" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="1">
+    <row r="4" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="1">
+    <row r="5" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="1">
+    <row r="6" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="1">
+    <row r="7" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="2" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="1">
+    <row r="8" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="1">
+    <row r="9" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="1">
+    <row r="10" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="1">
+    <row r="11" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="2" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="1">
+    <row r="12" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="2" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="1">
+    <row r="13" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="2" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="1">
+    <row r="14" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="2" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="1">
+    <row r="15" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="2" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="1">
+    <row r="16" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="1">
+    <row r="17" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="2" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="1">
+    <row r="18" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="1">
+    <row r="19" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="2" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="1">
+    <row r="20" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="2" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="1">
+    <row r="21" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="1">
+    <row r="22" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="2" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="1">
+    <row r="23" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="1">
+    <row r="24" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
         <v>23</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="2" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="1">
+    <row r="25" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="2" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="1">
+    <row r="26" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="2" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="1">
+    <row r="27" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="2" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="1">
+    <row r="28" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="2" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="1">
+    <row r="29" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="2" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="1">
+    <row r="30" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="2" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="1">
+    <row r="31" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="2" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="1">
+    <row r="32" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="2" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="1">
+    <row r="33" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="2" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="1">
+    <row r="34" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="2" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="1">
+    <row r="35" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="2" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="1">
+    <row r="36" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="2" t="s">
         <v>331</v>
       </c>
     </row>
@@ -4093,15 +4057,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="44.53125" customWidth="1"/>
     <col min="2" max="2" width="17.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>332</v>
       </c>
@@ -4109,7 +4073,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>334</v>
       </c>
@@ -4117,7 +4081,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>336</v>
       </c>
@@ -4125,7 +4089,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>338</v>
       </c>
@@ -4133,7 +4097,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>340</v>
       </c>
@@ -4141,7 +4105,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>342</v>
       </c>
@@ -4149,7 +4113,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>344</v>
       </c>
@@ -4163,86 +4127,60 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" style="19" customWidth="1"/>
-    <col min="2" max="2" width="25" style="19" customWidth="1"/>
-    <col min="3" max="3" width="20" style="19" customWidth="1"/>
-    <col min="4" max="4" width="45" style="19" customWidth="1"/>
-    <col min="5" max="5" width="80" style="20" customWidth="1"/>
-    <col min="6" max="6" width="45" style="19" customWidth="1"/>
+    <col min="1" max="1" width="30" style="20" customWidth="1"/>
+    <col min="2" max="2" width="25" style="20" customWidth="1"/>
+    <col min="3" max="3" width="20" style="20" customWidth="1"/>
+    <col min="4" max="4" width="45" style="20" customWidth="1"/>
+    <col min="5" max="5" width="80" style="21" customWidth="1"/>
+    <col min="6" max="6" width="45" style="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:6" s="22" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="24" t="s">
         <v>347</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="23" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="19" t="s">
-        <v>348</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" s="19" t="str">
-        <f>ประเมินผลทีม!A6</f>
-        <v>กฤษณพงศ์ ดลจิตต์</v>
-      </c>
-      <c r="B5" s="19" t="str">
-        <f>ประเมินผลทีม!B6</f>
-        <v>เจ้าหน้าที่บริการฯ</v>
-      </c>
-      <c r="C5" s="19" t="str">
-        <f>SUBSTITUTE(TRIM(IF((ประเมินผลทีม!D6+0.05)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," AGI","")&amp;IF((ประเมินผลทีม!G6+0.02)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," CON","")&amp;IF((ประเมินผลทีม!E6+0.04)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," DEX","")&amp;IF((ประเมินผลทีม!F6+0.03)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," INT","")&amp;IF((ประเมินผลทีม!H6+0.01)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," SEN","")&amp;IF((ประเมินผลทีม!C6+0.06)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},ประเมินผลทีม!C6,ประเมินผลทีม!D6,ประเมินผลทีม!E6,ประเมินผลทีม!F6,ประเมินผลทีม!G6,ประเมินผลทีม!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},(ประเมินผลทีม!C6+0.06),(ประเมินผลทีม!D6+0.05),(ประเมินผลทีม!E6+0.04),(ประเมินผลทีม!F6+0.03),(ประเมินผลทีม!G6+0.02),(ประเมินผลทีม!H6+0.01)),2))," STR",""))," ","+")</f>
-        <v>INT+SEN+STR</v>
-      </c>
-      <c r="D5" s="19" t="str">
-        <f>INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0))</f>
-        <v>Mastermind Overseer (สายผู้บงการเบ็ดเสร็จ)</v>
-      </c>
-      <c r="E5" s="20" t="str">
-        <f>INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0))</f>
-        <v>วิเคราะห์, จัดระบบ, ส่งมอบงานยาก: ผู้บงการเบื้องหลัง ใช้ Automation ประเมินสถานการณ์ แล้วสั่งการเคลียร์เคสพิพาทด้วยข้อมูลและเด็ดขาด</v>
-      </c>
-      <c r="F5" s="19" t="str">
-        <f>INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0))</f>
-        <v>The Almighty (ผู้ควบคุมทิศทางเบ็ดเสร็จ)</v>
+      <c r="C2" s="20" t="s">
+        <v>329</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>331</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Embed Growth Tendency logic as native Excel formulas in summary sheet
</commit_message>
<xml_diff>
--- a/rpg-performance-tracker-v6.xlsx
+++ b/rpg-performance-tracker-v6.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="4" activeTab="5"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="คำแนะนำการใช้งาน" state="visible" r:id="rId4"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="350">
   <si>
     <t>คู่มือและระบบบันทึกคะแนน RPG Status Framework (ฉบับอัปเดตเกณฑ์ใหม่)</t>
   </si>
@@ -227,6 +227,12 @@
   <si>
     <t xml:space="preserve">SEN3
 เทคโนโลยีลดขั้นตอน</t>
+  </si>
+  <si>
+    <t>นัชานันท์ ดิษฐวัฒน์วรกุล</t>
+  </si>
+  <si>
+    <t>ธุรการ</t>
   </si>
   <si>
     <t>กฤษณพงศ์ ดลจิตต์</t>
@@ -1137,6 +1143,8 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1944,127 +1952,121 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s">
+        <v>64</v>
+      </c>
       <c r="C3">
-        <f t="shared" ref="C3:C25" si="0">ROUND(ROUND(AVERAGE(K3:M3), 1), 0)</f>
-        <v>7</v>
+        <f t="shared" ref="C3:C25" si="2">ROUND(ROUND(AVERAGE(K3:M3), 1), 0)</f>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D25" si="1">ROUND(ROUND(AVERAGE(N3:P3), 1), 0)</f>
-        <v>7</v>
+        <f t="shared" ref="D3:D25" si="3">ROUND(ROUND(AVERAGE(N3:P3), 1), 0)</f>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E25" si="2">ROUND(ROUND(AVERAGE(Q3:S3), 1), 0)</f>
-        <v>8</v>
+        <f t="shared" ref="E3:E25" si="4">ROUND(ROUND(AVERAGE(Q3:S3), 1), 0)</f>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F25" si="3">ROUND(ROUND(AVERAGE(T3:W3), 1), 0)</f>
-        <v>7</v>
+        <f t="shared" ref="F3:F25" si="5">ROUND(ROUND(AVERAGE(T3:W3), 1), 0)</f>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G25" si="4">ROUND(ROUND(AVERAGE(X3:Z3), 1), 0)</f>
-        <v>6</v>
+        <f t="shared" ref="G3:G25" si="6">ROUND(ROUND(AVERAGE(X3:Z3), 1), 0)</f>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H25" si="5">ROUND(ROUND(AVERAGE(AA3:AC3), 1), 0)</f>
-        <v>7</v>
+        <f t="shared" ref="H3:H25" si="7">ROUND(ROUND(AVERAGE(AA3:AC3), 1), 0)</f>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I25" si="6">INDEX($C$2:$H$2, MATCH(MAX(C3:H3), C3:H3, 0))</f>
+        <f t="shared" ref="I3:I25" si="0">INDEX($C$2:$H$2, MATCH(MAX(C3:H3), C3:H3, 0))</f>
+        <v>STR เฉลี่ย</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J25" si="1">INDEX($C$2:$H$2, MATCH(MIN(C3:H3), C3:H3, 0))</f>
         <v>DEX เฉลี่ย</v>
       </c>
-      <c r="J3" t="str">
-        <f t="shared" ref="J3:J25" si="7">INDEX($C$2:$H$2, MATCH(MIN(C3:H3), C3:H3, 0))</f>
-        <v>CON เฉลี่ย</v>
-      </c>
       <c r="K3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N3">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P3">
+        <v>4</v>
+      </c>
+      <c r="Q3">
         <v>5</v>
       </c>
-      <c r="Q3">
-        <v>8</v>
-      </c>
       <c r="R3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="X3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Y3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z3">
         <v>6</v>
       </c>
       <c r="AA3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AB3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AC3">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C4">
         <f>ROUND(ROUND(AVERAGE(K4:M4), 1), 0)</f>
-        <v>5</v>
       </c>
       <c r="D4">
         <f>ROUND(ROUND(AVERAGE(N4:P4), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="E4">
         <f>ROUND(ROUND(AVERAGE(Q4:S4), 1), 0)</f>
-        <v>8</v>
       </c>
       <c r="F4">
         <f>ROUND(ROUND(AVERAGE(T4:W4), 1), 0)</f>
-        <v>5</v>
       </c>
       <c r="G4">
         <f>ROUND(ROUND(AVERAGE(X4:Z4), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="H4">
         <f>ROUND(ROUND(AVERAGE(AA4:AC4), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="I4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>DEX เฉลี่ย</v>
       </c>
       <c r="J4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="1"/>
         <v>STR เฉลี่ย</v>
       </c>
       <c r="K4">
@@ -2128,34 +2130,28 @@
     <row r="5" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C5">
         <f>ROUND(ROUND(AVERAGE(K5:M5), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="D5">
         <f>ROUND(ROUND(AVERAGE(N5:P5), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="E5">
         <f>ROUND(ROUND(AVERAGE(Q5:S5), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="F5">
         <f>ROUND(ROUND(AVERAGE(T5:W5), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="G5">
         <f>ROUND(ROUND(AVERAGE(X5:Z5), 1), 0)</f>
-        <v>8</v>
       </c>
       <c r="H5">
         <f>ROUND(ROUND(AVERAGE(AA5:AC5), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="I5" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>CON เฉลี่ย</v>
       </c>
       <c r="J5" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="1"/>
         <v>STR เฉลี่ย</v>
       </c>
       <c r="K5">
@@ -2218,41 +2214,35 @@
     </row>
     <row r="6" ht="15.75" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6">
         <f>ROUND(ROUND(AVERAGE(K6:M6), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="D6">
         <f>ROUND(ROUND(AVERAGE(N6:P6), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="E6">
         <f>ROUND(ROUND(AVERAGE(Q6:S6), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="F6">
         <f>ROUND(ROUND(AVERAGE(T6:W6), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="G6">
         <f>ROUND(ROUND(AVERAGE(X6:Z6), 1), 0)</f>
-        <v>6</v>
       </c>
       <c r="H6">
         <f>ROUND(ROUND(AVERAGE(AA6:AC6), 1), 0)</f>
-        <v>7</v>
       </c>
       <c r="I6" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>STR เฉลี่ย</v>
       </c>
       <c r="J6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="1"/>
         <v>AGI เฉลี่ย</v>
       </c>
       <c r="K6">
@@ -2315,647 +2305,647 @@
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D7" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E7" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F7" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G7" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H7" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I7" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D7" t="e">
+      <c r="J7" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F7" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G7" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I7" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J7" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C8" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D8" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E8" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F8" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G8" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H8" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I8" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D8" t="e">
+      <c r="J8" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F8" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G8" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H8" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I8" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J8" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D9" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E9" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F9" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G9" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H9" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D9" t="e">
+      <c r="J9" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E9" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F9" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G9" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I9" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J9" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D10" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E10" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F10" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G10" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I10" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D10" t="e">
+      <c r="J10" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E10" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F10" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G10" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H10" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I10" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J10" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C11" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D11" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E11" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F11" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G11" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H11" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I11" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D11" t="e">
+      <c r="J11" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E11" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F11" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G11" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H11" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I11" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J11" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D12" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E12" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F12" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G12" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H12" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I12" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D12" t="e">
+      <c r="J12" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E12" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F12" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G12" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H12" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I12" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J12" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C13" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D13" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E13" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F13" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G13" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H13" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I13" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D13" t="e">
+      <c r="J13" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E13" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F13" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H13" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I13" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J13" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C14" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D14" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E14" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F14" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G14" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H14" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I14" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D14" t="e">
+      <c r="J14" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E14" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F14" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G14" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H14" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I14" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J14" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C15" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D15" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E15" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F15" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G15" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H15" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I15" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D15" t="e">
+      <c r="J15" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E15" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F15" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G15" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H15" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I15" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J15" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C16" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D16" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E16" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F16" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G16" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H16" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I16" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D16" t="e">
+      <c r="J16" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E16" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F16" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G16" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H16" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I16" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J16" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C17" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D17" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E17" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F17" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G17" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H17" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I17" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D17" t="e">
+      <c r="J17" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E17" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F17" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G17" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H17" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I17" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J17" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C18" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D18" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E18" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F18" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G18" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H18" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D18" t="e">
+      <c r="J18" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E18" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F18" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G18" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H18" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I18" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J18" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C19" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D19" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E19" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F19" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G19" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H19" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I19" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D19" t="e">
+      <c r="J19" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E19" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F19" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G19" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H19" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I19" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J19" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C20" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D20" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E20" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F20" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G20" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H20" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I20" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D20" t="e">
+      <c r="J20" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E20" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F20" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G20" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H20" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I20" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J20" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C21" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D21" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E21" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F21" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G21" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H21" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I21" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D21" t="e">
+      <c r="J21" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E21" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F21" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G21" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I21" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J21" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C22" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D22" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E22" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F22" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G22" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H22" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I22" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D22" t="e">
+      <c r="J22" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E22" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F22" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G22" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H22" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I22" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J22" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C23" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D23" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E23" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F23" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G23" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H23" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I23" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D23" t="e">
+      <c r="J23" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E23" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F23" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G23" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H23" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I23" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J23" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C24" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D24" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E24" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F24" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G24" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H24" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I24" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D24" t="e">
+      <c r="J24" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E24" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F24" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G24" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H24" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I24" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C25" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D25" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E25" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F25" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G25" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H25" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I25" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D25" t="e">
+      <c r="J25" t="e">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E25" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F25" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G25" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H25" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I25" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J25" t="e">
-        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2983,7 +2973,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2994,423 +2984,423 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="20" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3441,19 +3431,19 @@
   <sheetData>
     <row r="1" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3461,16 +3451,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3478,16 +3468,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3495,16 +3485,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3512,16 +3502,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3529,16 +3519,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3546,16 +3536,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3563,16 +3553,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3580,16 +3570,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3597,16 +3587,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3614,16 +3604,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3631,16 +3621,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3648,16 +3638,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="14" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3665,16 +3655,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3682,16 +3672,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3699,16 +3689,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3716,16 +3706,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="18" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3733,16 +3723,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3750,16 +3740,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3767,16 +3757,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3784,16 +3774,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3801,16 +3791,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3818,16 +3808,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3835,16 +3825,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3852,16 +3842,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3869,16 +3859,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3886,16 +3876,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="28" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3903,16 +3893,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="29" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3920,16 +3910,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="30" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3937,16 +3927,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="31" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3954,16 +3944,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="32" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3971,16 +3961,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="33" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3988,16 +3978,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="34" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4005,16 +3995,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="35" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4022,16 +4012,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="36" ht="80" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4039,16 +4029,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -4067,58 +4057,58 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B4" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B6" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B7" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -4128,8 +4118,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30" style="20" customWidth="1"/>
     <col min="2" max="2" width="25" style="20" customWidth="1"/>
@@ -4147,40 +4137,60 @@
         <v>35</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>329</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>328</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>331</v>
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" ht="28.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="20">
+        <f>'ประเมินผลทีม'!A3</f>
+      </c>
+      <c r="B2" s="20">
+        <f>'ประเมินผลทีม'!B3</f>
+      </c>
+      <c r="C2" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, "Growth Tendency", SUBSTITUTE(TRIM(IF(('ประเมินผลทีม'!D3+0.05)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," AGI","")&amp;IF(('ประเมินผลทีม'!G3+0.02)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," CON","")&amp;IF(('ประเมินผลทีม'!E3+0.04)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," DEX","")&amp;IF(('ประเมินผลทีม'!F3+0.03)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," INT","")&amp;IF(('ประเมินผลทีม'!H3+0.01)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," SEN","")&amp;IF(('ประเมินผลทีม'!C3+0.06)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," STR",""))," ","+"))</f>
+      </c>
+      <c r="D2" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer (ผู้ประคองงาน)", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention (ผู้ต้องได้รับการดูแล)", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "Apprentice (ผู้ฝึกหัด)", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", TRUE, "Uncalibrated (ศักยภาพที่รอการเจียระไน)"), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+      </c>
+      <c r="E2" s="21">
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", TRUE, "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น"), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+      </c>
+      <c r="F2" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "The Standard", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Undeveloped Potential", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "The Beginner", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Emerging Talent", TRUE, "Uncalibrated"), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="20">
+        <f>'ประเมินผลทีม'!A6</f>
+      </c>
+      <c r="B5" s="20">
+        <f>'ประเมินผลทีม'!B6</f>
+      </c>
+      <c r="C5" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, "Growth Tendency", SUBSTITUTE(TRIM(IF(('ประเมินผลทีม'!D6+0.05)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," AGI","")&amp;IF(('ประเมินผลทีม'!G6+0.02)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," CON","")&amp;IF(('ประเมินผลทีม'!E6+0.04)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," DEX","")&amp;IF(('ประเมินผลทีม'!F6+0.03)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," INT","")&amp;IF(('ประเมินผลทีม'!H6+0.01)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," SEN","")&amp;IF(('ประเมินผลทีม'!C6+0.06)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," STR",""))," ","+"))</f>
+      </c>
+      <c r="D5" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer (ผู้ประคองงาน)", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention (ผู้ต้องได้รับการดูแล)", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "Apprentice (ผู้ฝึกหัด)", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", TRUE, "Uncalibrated (ศักยภาพที่รอการเจียระไน)"), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", TRUE, "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น"), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+      </c>
+      <c r="F5" s="20">
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "The Standard", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Undeveloped Potential", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "The Beginner", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Emerging Talent", TRUE, "Uncalibrated"), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update v6 Excel with nested IF formula for older Excel compatibility
</commit_message>
<xml_diff>
--- a/rpg-performance-tracker-v6.xlsx
+++ b/rpg-performance-tracker-v6.xlsx
@@ -4160,13 +4160,13 @@
         <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, "Growth Tendency", SUBSTITUTE(TRIM(IF(('ประเมินผลทีม'!D3+0.05)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," AGI","")&amp;IF(('ประเมินผลทีม'!G3+0.02)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," CON","")&amp;IF(('ประเมินผลทีม'!E3+0.04)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," DEX","")&amp;IF(('ประเมินผลทีม'!F3+0.03)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," INT","")&amp;IF(('ประเมินผลทีม'!H3+0.01)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," SEN","")&amp;IF(('ประเมินผลทีม'!C3+0.06)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C3,'ประเมินผลทีม'!D3,'ประเมินผลทีม'!E3,'ประเมินผลทีม'!F3,'ประเมินผลทีม'!G3,'ประเมินผลทีม'!H3),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C3+0.06),('ประเมินผลทีม'!D3+0.05),('ประเมินผลทีม'!E3+0.04),('ประเมินผลทีม'!F3+0.03),('ประเมินผลทีม'!G3+0.02),('ประเมินผลทีม'!H3+0.01)),2))," STR",""))," ","+"))</f>
       </c>
       <c r="D2" s="20">
-        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer (ผู้ประคองงาน)", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention (ผู้ต้องได้รับการดูแล)", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "Apprentice (ผู้ฝึกหัด)", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", TRUE, "Uncalibrated (ศักยภาพที่รอการเจียระไน)"), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", IF(AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer (ผู้ประคองงาน)", IF(AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention (ผู้ต้องได้รับการดูแล)", IF(MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "Apprentice (ผู้ฝึกหัด)", IF(AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", "Uncalibrated (ศักยภาพที่รอการเจียระไน)")))))), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
       <c r="E2" s="21">
-        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", TRUE, "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น"), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", IF(AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", IF(AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", IF(MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", IF(AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น")))))), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
       <c r="F2" s="20">
-        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "The Standard", AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer", AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention", MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Undeveloped Potential", MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "The Beginner", AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Emerging Talent", TRUE, "Uncalibrated"), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C3:H3)=5, MIN('ประเมินผลทีม'!C3:H3)=5), "The Standard", IF(AND(MAX('ประเมินผลทีม'!C3:H3)=4, MIN('ประเมินผลทีม'!C3:H3)=4), "The Maintainer", IF(AND(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, MIN('ประเมินผลทีม'!C3:H3)=MAX('ประเมินผลทีม'!C3:H3)), "Needs Attention", IF(MIN('ประเมินผลทีม'!C3:H3)&gt;=4, "Undeveloped Potential", IF(MAX('ประเมินผลทีม'!C3:H3)&lt;=3, "The Beginner", IF(AND(COUNTIF('ประเมินผลทีม'!C3:H3, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C3:H3, "&lt;=3")&gt;0), "Emerging Talent", "Uncalibrated")))))), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C2, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -4180,13 +4180,13 @@
         <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, "Growth Tendency", SUBSTITUTE(TRIM(IF(('ประเมินผลทีม'!D6+0.05)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," AGI","")&amp;IF(('ประเมินผลทีม'!G6+0.02)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," CON","")&amp;IF(('ประเมินผลทีม'!E6+0.04)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," DEX","")&amp;IF(('ประเมินผลทีม'!F6+0.03)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," INT","")&amp;IF(('ประเมินผลทีม'!H6+0.01)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," SEN","")&amp;IF(('ประเมินผลทีม'!C6+0.06)&gt;=IF(LARGE(CHOOSE({1,2,3,4,5,6},'ประเมินผลทีม'!C6,'ประเมินผลทีม'!D6,'ประเมินผลทีม'!E6,'ประเมินผลทีม'!F6,'ประเมินผลทีม'!G6,'ประเมินผลทีม'!H6),3)&gt;=6.5,LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),3),LARGE(CHOOSE({1,2,3,4,5,6},('ประเมินผลทีม'!C6+0.06),('ประเมินผลทีม'!D6+0.05),('ประเมินผลทีม'!E6+0.04),('ประเมินผลทีม'!F6+0.03),('ประเมินผลทีม'!G6+0.02),('ประเมินผลทีม'!H6+0.01)),2))," STR",""))," ","+"))</f>
       </c>
       <c r="D5" s="20">
-        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer (ผู้ประคองงาน)", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention (ผู้ต้องได้รับการดูแล)", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "Apprentice (ผู้ฝึกหัด)", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", TRUE, "Uncalibrated (ศักยภาพที่รอการเจียระไน)"), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "Standard Achiever (ผู้บรรลุมาตรฐาน)", IF(AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer (ผู้ประคองงาน)", IF(AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention (ผู้ต้องได้รับการดูแล)", IF(MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Generalist (ผู้เรียนรู้รอบด้าน)", IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "Apprentice (ผู้ฝึกหัด)", IF(AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Rookie (ดาวรุ่ง)", "Uncalibrated (ศักยภาพที่รอการเจียระไน)")))))), INDEX('Archetypes Guide V2'!$B$2:$B$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
       <c r="E5" s="21">
-        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", TRUE, "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น"), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "ปฏิบัติงานได้ตามมาตรฐานอย่างครบถ้วนในทุกมิติ เป็นฟันเฟืองที่พึ่งพาได้ ควรกล้ารับความท้าทายใหม่ๆ เพื่อยกระดับสู่ผู้เชี่ยวชาญ", IF(AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "ประคองการทำงานภาพรวมได้ แต่มีช่องโหว่ในรายละเอียด ควรเน้นความรอบคอบและเรียนรู้จากพี่เลี้ยงเพื่อยกระดับผลงาน", IF(AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "ผลการปฏิบัติงานต่ำกว่าเกณฑ์ในทุกมิติ หัวหน้างานควรเร่งประเมินสาเหตุและวางแผนปรับพื้นฐานใหม่ (Re-train) อย่างเร่งด่วน", IF(MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "มีพื้นฐานที่สม่ำเสมอและปรับตัวได้ทุกบทบาท ควรผลักดันให้หา ""ความถนัดเฉพาะทาง"" 1-2 ด้าน เพื่อทะลุกำแพงสู่ระดับที่สูงขึ้น", IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "อยู่ในช่วงเริ่มต้นหรือยังไม่คุ้นเคยกับกระบวนการ ต้องการการสอนงานอย่างใกล้ชิด (OJT) และกำหนดเป้าหมายที่ชัดเจน", IF(AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "เริ่มฉายแววในด้านที่ถนัด แต่ทักษะอื่นยังไม่เสถียร ควรส่งเสริมจุดแข็งและใช้พี่เลี้ยงประคองจุดอ่อน", "ศักยภาพแฝงมีแต่ผลงานยังขาดความสม่ำเสมอ หัวหน้าควรช่วยจัดลำดับความสำคัญและแก้จุดอ่อนทีละจุดเพื่อให้ผลงานนิ่งขึ้น")))))), INDEX('Archetypes Guide V2'!$D$2:$D$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
       <c r="F5" s="20">
-        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IFS(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "The Standard", AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer", AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention", MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Undeveloped Potential", MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "The Beginner", AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Emerging Talent", TRUE, "Uncalibrated"), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
+        <f>IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=5, IF(AND(MAX('ประเมินผลทีม'!C6:H6)=5, MIN('ประเมินผลทีม'!C6:H6)=5), "The Standard", IF(AND(MAX('ประเมินผลทีม'!C6:H6)=4, MIN('ประเมินผลทีม'!C6:H6)=4), "The Maintainer", IF(AND(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, MIN('ประเมินผลทีม'!C6:H6)=MAX('ประเมินผลทีม'!C6:H6)), "Needs Attention", IF(MIN('ประเมินผลทีม'!C6:H6)&gt;=4, "Undeveloped Potential", IF(MAX('ประเมินผลทีม'!C6:H6)&lt;=3, "The Beginner", IF(AND(COUNTIF('ประเมินผลทีม'!C6:H6, "&gt;=4")&gt;0, COUNTIF('ประเมินผลทีม'!C6:H6, "&lt;=3")&gt;0), "Emerging Talent", "Uncalibrated")))))), INDEX('Archetypes Guide V2'!$E$2:$E$36, MATCH(C5, 'Archetypes Guide V2'!$C$2:$C$36, 0)))</f>
       </c>
     </row>
   </sheetData>

</xml_diff>